<commit_message>
working my way to report generation, almost there
</commit_message>
<xml_diff>
--- a/Timesheeter/Timesheet_Template_Excel/Timesheet.xlsx
+++ b/Timesheeter/Timesheet_Template_Excel/Timesheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\source\repos\Timesheet_App\Timesheeter\Timesheet_Template_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E755BEB-AEB7-4D0C-8DA6-2B5B85127C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3AB7FB4-CE95-4387-ACCA-718F2638F8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,22 +18,22 @@
   <definedNames>
     <definedName name="Customer" localSheetId="0">CW!$C$2</definedName>
     <definedName name="Customer">#REF!</definedName>
-    <definedName name="DailyActivityDescriptionFriday">CW!$I$36:$O$40</definedName>
-    <definedName name="DailyActivityDescriptionMonday">CW!$I$16:$O$20</definedName>
-    <definedName name="DailyActivityDescriptionSaturday">CW!$I$41:$O$45</definedName>
-    <definedName name="DailyActivityDescriptionSunday">CW!$I$46:$O$49</definedName>
-    <definedName name="DailyActivityDescriptionThursday">CW!$I$31:$O$35</definedName>
-    <definedName name="DailyActivityDescriptionTuesday">CW!$I$21:$O$25</definedName>
-    <definedName name="DailyActivityDescriptionWednesday">CW!$I$26:$O$30</definedName>
+    <definedName name="DailyActivityDescriptionFriday" localSheetId="0">CW!$I$36:$O$40</definedName>
+    <definedName name="DailyActivityDescriptionMonday" localSheetId="0">CW!$I$16:$O$20</definedName>
+    <definedName name="DailyActivityDescriptionSaturday" localSheetId="0">CW!$I$41:$O$45</definedName>
+    <definedName name="DailyActivityDescriptionSunday" localSheetId="0">CW!$I$46:$O$49</definedName>
+    <definedName name="DailyActivityDescriptionThursday" localSheetId="0">CW!$I$31:$O$35</definedName>
+    <definedName name="DailyActivityDescriptionTuesday" localSheetId="0">CW!$I$21:$O$25</definedName>
+    <definedName name="DailyActivityDescriptionWednesday" localSheetId="0">CW!$I$26:$O$30</definedName>
     <definedName name="Engineer" localSheetId="0">CW!$K$2</definedName>
     <definedName name="Engineer">#REF!</definedName>
-    <definedName name="HoursFriday">CW!$D$38</definedName>
-    <definedName name="HoursMonday">CW!$D$18</definedName>
-    <definedName name="HoursSaturday">CW!$D$43</definedName>
-    <definedName name="HoursSunday">CW!$D$48</definedName>
-    <definedName name="HoursThursday">CW!$D$33</definedName>
-    <definedName name="HoursTuesday">CW!$D$23</definedName>
-    <definedName name="HoursWednesday">CW!$D$28</definedName>
+    <definedName name="HoursFriday" localSheetId="0">CW!$D$38</definedName>
+    <definedName name="HoursMonday" localSheetId="0">CW!$D$18</definedName>
+    <definedName name="HoursSaturday" localSheetId="0">CW!$D$43</definedName>
+    <definedName name="HoursSunday" localSheetId="0">CW!$D$48</definedName>
+    <definedName name="HoursThursday" localSheetId="0">CW!$D$33</definedName>
+    <definedName name="HoursTuesday" localSheetId="0">CW!$D$23</definedName>
+    <definedName name="HoursWednesday" localSheetId="0">CW!$D$28</definedName>
     <definedName name="Location" localSheetId="0">CW!$C$4</definedName>
     <definedName name="Location">#REF!</definedName>
     <definedName name="ProjLineName" localSheetId="0">CW!$C$6</definedName>
@@ -41,7 +41,7 @@
     <definedName name="ProjNumber">CW!$L$4</definedName>
     <definedName name="Purpose" localSheetId="0">CW!$C$8</definedName>
     <definedName name="Purpose">#REF!</definedName>
-    <definedName name="Start_Date">CW!$B$18</definedName>
+    <definedName name="Start_Date" localSheetId="0">CW!$B$18</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -655,6 +655,69 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -663,69 +726,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1138,14 +1138,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
     </row>
     <row r="2" spans="2:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
@@ -1167,11 +1167,11 @@
         <v>3</v>
       </c>
       <c r="D4" s="3"/>
-      <c r="I4" s="48" t="s">
+      <c r="I4" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
     </row>
     <row r="6" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
@@ -1187,19 +1187,19 @@
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="47"/>
-      <c r="J8" s="47"/>
-      <c r="K8" s="47"/>
-      <c r="L8" s="47"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="47"/>
-      <c r="O8" s="47"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="68"/>
+      <c r="I8" s="68"/>
+      <c r="J8" s="68"/>
+      <c r="K8" s="68"/>
+      <c r="L8" s="68"/>
+      <c r="M8" s="68"/>
+      <c r="N8" s="68"/>
+      <c r="O8" s="68"/>
       <c r="P8" s="5"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.2">
@@ -1214,35 +1214,35 @@
       <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="47"/>
-      <c r="M10" s="47"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="47"/>
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="68"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="68"/>
+      <c r="J10" s="68"/>
+      <c r="K10" s="68"/>
+      <c r="L10" s="68"/>
+      <c r="M10" s="68"/>
+      <c r="N10" s="68"/>
+      <c r="O10" s="68"/>
       <c r="P10" s="5"/>
     </row>
     <row r="12" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="47"/>
+      <c r="C12" s="68"/>
+      <c r="D12" s="68"/>
+      <c r="E12" s="68"/>
+      <c r="F12" s="68"/>
+      <c r="G12" s="68"/>
+      <c r="H12" s="68"/>
+      <c r="I12" s="68"/>
+      <c r="J12" s="68"/>
+      <c r="K12" s="68"/>
+      <c r="L12" s="68"/>
+      <c r="M12" s="68"/>
+      <c r="N12" s="68"/>
+      <c r="O12" s="68"/>
       <c r="P12" s="5"/>
     </row>
     <row r="14" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -1273,15 +1273,15 @@
       <c r="H15" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="I15" s="60" t="s">
+      <c r="I15" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="J15" s="60"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="61"/>
+      <c r="J15" s="63"/>
+      <c r="K15" s="63"/>
+      <c r="L15" s="63"/>
+      <c r="M15" s="63"/>
+      <c r="N15" s="63"/>
+      <c r="O15" s="64"/>
       <c r="P15" s="6"/>
     </row>
     <row r="16" spans="2:16" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1294,13 +1294,13 @@
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="52"/>
-      <c r="N16" s="52"/>
-      <c r="O16" s="52"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="55"/>
+      <c r="N16" s="55"/>
+      <c r="O16" s="55"/>
       <c r="P16" s="8"/>
     </row>
     <row r="17" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1311,13 +1311,13 @@
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="53"/>
-      <c r="K17" s="53"/>
-      <c r="L17" s="53"/>
-      <c r="M17" s="53"/>
-      <c r="N17" s="53"/>
-      <c r="O17" s="54"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="50"/>
       <c r="P17" s="6"/>
     </row>
     <row r="18" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1327,13 +1327,13 @@
       <c r="E18" s="34"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
-      <c r="I18" s="49"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="50"/>
-      <c r="M18" s="50"/>
-      <c r="N18" s="50"/>
-      <c r="O18" s="55"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="47"/>
+      <c r="M18" s="47"/>
+      <c r="N18" s="47"/>
+      <c r="O18" s="61"/>
       <c r="P18" s="6"/>
     </row>
     <row r="19" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1344,13 +1344,13 @@
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" s="44"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
-      <c r="M19" s="53"/>
-      <c r="N19" s="53"/>
-      <c r="O19" s="56"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="49"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="57"/>
       <c r="Q19" s="43"/>
     </row>
     <row r="20" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -1361,13 +1361,13 @@
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
       <c r="H20" s="11"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="57"/>
-      <c r="M20" s="57"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="58"/>
+      <c r="I20" s="65"/>
+      <c r="J20" s="65"/>
+      <c r="K20" s="65"/>
+      <c r="L20" s="65"/>
+      <c r="M20" s="65"/>
+      <c r="N20" s="65"/>
+      <c r="O20" s="66"/>
       <c r="Q20" s="43"/>
     </row>
     <row r="21" spans="2:17" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1380,13 +1380,13 @@
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="53"/>
-      <c r="L21" s="53"/>
-      <c r="M21" s="53"/>
-      <c r="N21" s="53"/>
-      <c r="O21" s="54"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="50"/>
       <c r="P21" s="8"/>
     </row>
     <row r="22" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1396,13 +1396,13 @@
       <c r="E22" s="34"/>
       <c r="F22" s="42"/>
       <c r="H22" s="42"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="50"/>
-      <c r="K22" s="50"/>
-      <c r="L22" s="50"/>
-      <c r="M22" s="50"/>
-      <c r="N22" s="50"/>
-      <c r="O22" s="55"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="47"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="61"/>
       <c r="P22" s="6"/>
     </row>
     <row r="23" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1416,13 +1416,13 @@
       <c r="F23" s="6"/>
       <c r="G23" s="34"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="53"/>
-      <c r="K23" s="53"/>
-      <c r="L23" s="53"/>
-      <c r="M23" s="53"/>
-      <c r="N23" s="53"/>
-      <c r="O23" s="56"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="49"/>
+      <c r="N23" s="49"/>
+      <c r="O23" s="57"/>
       <c r="P23" s="6"/>
     </row>
     <row r="24" spans="2:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1433,13 +1433,13 @@
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="50"/>
-      <c r="K24" s="50"/>
-      <c r="L24" s="50"/>
-      <c r="M24" s="50"/>
-      <c r="N24" s="50"/>
-      <c r="O24" s="51"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="47"/>
+      <c r="M24" s="47"/>
+      <c r="N24" s="47"/>
+      <c r="O24" s="48"/>
       <c r="P24" s="6"/>
     </row>
     <row r="25" spans="2:17" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1450,13 +1450,13 @@
       <c r="F25" s="11"/>
       <c r="G25" s="11"/>
       <c r="H25" s="11"/>
-      <c r="I25" s="57"/>
-      <c r="J25" s="57"/>
-      <c r="K25" s="57"/>
-      <c r="L25" s="57"/>
-      <c r="M25" s="57"/>
-      <c r="N25" s="57"/>
-      <c r="O25" s="57"/>
+      <c r="I25" s="65"/>
+      <c r="J25" s="65"/>
+      <c r="K25" s="65"/>
+      <c r="L25" s="65"/>
+      <c r="M25" s="65"/>
+      <c r="N25" s="65"/>
+      <c r="O25" s="65"/>
       <c r="P25" s="6"/>
     </row>
     <row r="26" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -1469,13 +1469,13 @@
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
-      <c r="I26" s="52"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="52"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="55"/>
+      <c r="K26" s="55"/>
+      <c r="L26" s="55"/>
+      <c r="M26" s="55"/>
+      <c r="N26" s="55"/>
+      <c r="O26" s="55"/>
       <c r="P26" s="6"/>
     </row>
     <row r="27" spans="2:17" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1486,13 +1486,13 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="53"/>
-      <c r="L27" s="53"/>
-      <c r="M27" s="53"/>
-      <c r="N27" s="53"/>
-      <c r="O27" s="56"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="49"/>
+      <c r="L27" s="49"/>
+      <c r="M27" s="49"/>
+      <c r="N27" s="49"/>
+      <c r="O27" s="57"/>
       <c r="P27" s="8"/>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.2">
@@ -1505,13 +1505,13 @@
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="50"/>
-      <c r="L28" s="50"/>
-      <c r="M28" s="50"/>
-      <c r="N28" s="50"/>
-      <c r="O28" s="51"/>
+      <c r="I28" s="46"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="47"/>
+      <c r="N28" s="47"/>
+      <c r="O28" s="48"/>
       <c r="P28" s="6"/>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.2">
@@ -1521,13 +1521,13 @@
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
-      <c r="I29" s="49"/>
-      <c r="J29" s="50"/>
-      <c r="K29" s="50"/>
-      <c r="L29" s="50"/>
-      <c r="M29" s="50"/>
-      <c r="N29" s="50"/>
-      <c r="O29" s="51"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="47"/>
+      <c r="L29" s="47"/>
+      <c r="M29" s="47"/>
+      <c r="N29" s="47"/>
+      <c r="O29" s="48"/>
     </row>
     <row r="30" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B30" s="24"/>
@@ -1537,13 +1537,13 @@
       <c r="F30" s="11"/>
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
-      <c r="I30" s="62"/>
-      <c r="J30" s="63"/>
-      <c r="K30" s="63"/>
-      <c r="L30" s="63"/>
-      <c r="M30" s="63"/>
-      <c r="N30" s="63"/>
-      <c r="O30" s="64"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="52"/>
+      <c r="K30" s="52"/>
+      <c r="L30" s="52"/>
+      <c r="M30" s="52"/>
+      <c r="N30" s="52"/>
+      <c r="O30" s="53"/>
     </row>
     <row r="31" spans="2:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B31" s="23" t="s">
@@ -1555,13 +1555,13 @@
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
-      <c r="I31" s="52"/>
-      <c r="J31" s="52"/>
-      <c r="K31" s="52"/>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="52"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="55"/>
+      <c r="K31" s="55"/>
+      <c r="L31" s="55"/>
+      <c r="M31" s="55"/>
+      <c r="N31" s="55"/>
+      <c r="O31" s="55"/>
       <c r="P31" s="6"/>
     </row>
     <row r="32" spans="2:17" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1572,13 +1572,13 @@
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="53"/>
-      <c r="K32" s="53"/>
-      <c r="L32" s="53"/>
-      <c r="M32" s="53"/>
-      <c r="N32" s="53"/>
-      <c r="O32" s="54"/>
+      <c r="I32" s="46"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+      <c r="M32" s="49"/>
+      <c r="N32" s="49"/>
+      <c r="O32" s="50"/>
       <c r="P32" s="8"/>
     </row>
     <row r="33" spans="2:16" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -1592,13 +1592,13 @@
       <c r="F33" s="40"/>
       <c r="G33" s="41"/>
       <c r="H33" s="40"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="50"/>
-      <c r="K33" s="50"/>
-      <c r="L33" s="50"/>
-      <c r="M33" s="50"/>
-      <c r="N33" s="50"/>
-      <c r="O33" s="51"/>
+      <c r="I33" s="46"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="47"/>
+      <c r="L33" s="47"/>
+      <c r="M33" s="47"/>
+      <c r="N33" s="47"/>
+      <c r="O33" s="48"/>
       <c r="P33" s="6"/>
     </row>
     <row r="34" spans="2:16" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -1609,13 +1609,13 @@
       <c r="F34" s="17"/>
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
-      <c r="I34" s="49"/>
-      <c r="J34" s="50"/>
-      <c r="K34" s="50"/>
-      <c r="L34" s="50"/>
-      <c r="M34" s="50"/>
-      <c r="N34" s="50"/>
-      <c r="O34" s="51"/>
+      <c r="I34" s="46"/>
+      <c r="J34" s="47"/>
+      <c r="K34" s="47"/>
+      <c r="L34" s="47"/>
+      <c r="M34" s="47"/>
+      <c r="N34" s="47"/>
+      <c r="O34" s="48"/>
       <c r="P34" s="6"/>
     </row>
     <row r="35" spans="2:16" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1626,13 +1626,13 @@
       <c r="F35" s="11"/>
       <c r="G35" s="11"/>
       <c r="H35" s="11"/>
-      <c r="I35" s="62"/>
-      <c r="J35" s="63"/>
-      <c r="K35" s="63"/>
-      <c r="L35" s="63"/>
-      <c r="M35" s="63"/>
-      <c r="N35" s="63"/>
-      <c r="O35" s="64"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="52"/>
+      <c r="K35" s="52"/>
+      <c r="L35" s="52"/>
+      <c r="M35" s="52"/>
+      <c r="N35" s="52"/>
+      <c r="O35" s="53"/>
       <c r="P35" s="6"/>
     </row>
     <row r="36" spans="2:16" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1645,13 +1645,13 @@
       <c r="F36" s="7"/>
       <c r="G36" s="7"/>
       <c r="H36" s="7"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="L36" s="52"/>
-      <c r="M36" s="52"/>
-      <c r="N36" s="52"/>
-      <c r="O36" s="52"/>
+      <c r="I36" s="55"/>
+      <c r="J36" s="55"/>
+      <c r="K36" s="55"/>
+      <c r="L36" s="55"/>
+      <c r="M36" s="55"/>
+      <c r="N36" s="55"/>
+      <c r="O36" s="55"/>
       <c r="P36" s="6"/>
     </row>
     <row r="37" spans="2:16" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1677,13 +1677,13 @@
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="50"/>
-      <c r="K38" s="50"/>
-      <c r="L38" s="50"/>
-      <c r="M38" s="50"/>
-      <c r="N38" s="50"/>
-      <c r="O38" s="51"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="47"/>
+      <c r="K38" s="47"/>
+      <c r="L38" s="47"/>
+      <c r="M38" s="47"/>
+      <c r="N38" s="47"/>
+      <c r="O38" s="48"/>
       <c r="P38" s="6"/>
     </row>
     <row r="39" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1694,13 +1694,13 @@
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
-      <c r="I39" s="59"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="53"/>
-      <c r="L39" s="53"/>
-      <c r="M39" s="53"/>
-      <c r="N39" s="53"/>
-      <c r="O39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="49"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="49"/>
+      <c r="M39" s="49"/>
+      <c r="N39" s="49"/>
+      <c r="O39" s="57"/>
       <c r="P39" s="6"/>
     </row>
     <row r="40" spans="2:16" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1711,13 +1711,13 @@
       <c r="F40" s="11"/>
       <c r="G40" s="11"/>
       <c r="H40" s="11"/>
-      <c r="I40" s="66"/>
-      <c r="J40" s="67"/>
-      <c r="K40" s="67"/>
-      <c r="L40" s="67"/>
-      <c r="M40" s="67"/>
-      <c r="N40" s="67"/>
-      <c r="O40" s="68"/>
+      <c r="I40" s="58"/>
+      <c r="J40" s="59"/>
+      <c r="K40" s="59"/>
+      <c r="L40" s="59"/>
+      <c r="M40" s="59"/>
+      <c r="N40" s="59"/>
+      <c r="O40" s="60"/>
       <c r="P40" s="6"/>
     </row>
     <row r="41" spans="2:16" ht="13.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1730,13 +1730,13 @@
       <c r="F41" s="7"/>
       <c r="G41" s="7"/>
       <c r="H41" s="7"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="L41" s="52"/>
-      <c r="M41" s="52"/>
-      <c r="N41" s="52"/>
-      <c r="O41" s="52"/>
+      <c r="I41" s="55"/>
+      <c r="J41" s="55"/>
+      <c r="K41" s="55"/>
+      <c r="L41" s="55"/>
+      <c r="M41" s="55"/>
+      <c r="N41" s="55"/>
+      <c r="O41" s="55"/>
       <c r="P41" s="6"/>
     </row>
     <row r="42" spans="2:16" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1762,13 +1762,13 @@
       <c r="F43" s="7"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
-      <c r="I43" s="49"/>
-      <c r="J43" s="50"/>
-      <c r="K43" s="50"/>
-      <c r="L43" s="50"/>
-      <c r="M43" s="50"/>
-      <c r="N43" s="50"/>
-      <c r="O43" s="51"/>
+      <c r="I43" s="46"/>
+      <c r="J43" s="47"/>
+      <c r="K43" s="47"/>
+      <c r="L43" s="47"/>
+      <c r="M43" s="47"/>
+      <c r="N43" s="47"/>
+      <c r="O43" s="48"/>
       <c r="P43" s="6"/>
     </row>
     <row r="44" spans="2:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -1779,13 +1779,13 @@
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
-      <c r="I44" s="49"/>
-      <c r="J44" s="50"/>
-      <c r="K44" s="50"/>
-      <c r="L44" s="50"/>
-      <c r="M44" s="50"/>
-      <c r="N44" s="50"/>
-      <c r="O44" s="55"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="47"/>
+      <c r="K44" s="47"/>
+      <c r="L44" s="47"/>
+      <c r="M44" s="47"/>
+      <c r="N44" s="47"/>
+      <c r="O44" s="61"/>
       <c r="P44" s="6"/>
     </row>
     <row r="45" spans="2:16" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1796,13 +1796,13 @@
       <c r="F45" s="11"/>
       <c r="G45" s="11"/>
       <c r="H45" s="11"/>
-      <c r="I45" s="62"/>
-      <c r="J45" s="63"/>
-      <c r="K45" s="63"/>
-      <c r="L45" s="63"/>
-      <c r="M45" s="63"/>
-      <c r="N45" s="63"/>
-      <c r="O45" s="65"/>
+      <c r="I45" s="51"/>
+      <c r="J45" s="52"/>
+      <c r="K45" s="52"/>
+      <c r="L45" s="52"/>
+      <c r="M45" s="52"/>
+      <c r="N45" s="52"/>
+      <c r="O45" s="54"/>
       <c r="P45" s="6"/>
     </row>
     <row r="46" spans="2:16" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1815,13 +1815,13 @@
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
-      <c r="I46" s="52"/>
-      <c r="J46" s="52"/>
-      <c r="K46" s="52"/>
-      <c r="L46" s="52"/>
-      <c r="M46" s="52"/>
-      <c r="N46" s="52"/>
-      <c r="O46" s="69"/>
+      <c r="I46" s="55"/>
+      <c r="J46" s="55"/>
+      <c r="K46" s="55"/>
+      <c r="L46" s="55"/>
+      <c r="M46" s="55"/>
+      <c r="N46" s="55"/>
+      <c r="O46" s="62"/>
       <c r="P46" s="6"/>
     </row>
     <row r="47" spans="2:16" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1832,13 +1832,13 @@
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
-      <c r="I47" s="49"/>
-      <c r="J47" s="53"/>
-      <c r="K47" s="53"/>
-      <c r="L47" s="53"/>
-      <c r="M47" s="53"/>
-      <c r="N47" s="53"/>
-      <c r="O47" s="54"/>
+      <c r="I47" s="46"/>
+      <c r="J47" s="49"/>
+      <c r="K47" s="49"/>
+      <c r="L47" s="49"/>
+      <c r="M47" s="49"/>
+      <c r="N47" s="49"/>
+      <c r="O47" s="50"/>
       <c r="P47" s="8"/>
     </row>
     <row r="48" spans="2:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -1851,13 +1851,13 @@
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
-      <c r="I48" s="49"/>
-      <c r="J48" s="53"/>
-      <c r="K48" s="53"/>
-      <c r="L48" s="53"/>
-      <c r="M48" s="53"/>
-      <c r="N48" s="53"/>
-      <c r="O48" s="54"/>
+      <c r="I48" s="46"/>
+      <c r="J48" s="49"/>
+      <c r="K48" s="49"/>
+      <c r="L48" s="49"/>
+      <c r="M48" s="49"/>
+      <c r="N48" s="49"/>
+      <c r="O48" s="50"/>
       <c r="P48" s="6"/>
     </row>
     <row r="49" spans="2:16" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1868,13 +1868,13 @@
       <c r="F49" s="11"/>
       <c r="G49" s="11"/>
       <c r="H49" s="11"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="63"/>
-      <c r="K49" s="63"/>
-      <c r="L49" s="63"/>
-      <c r="M49" s="63"/>
-      <c r="N49" s="63"/>
-      <c r="O49" s="65"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="52"/>
+      <c r="K49" s="52"/>
+      <c r="L49" s="52"/>
+      <c r="M49" s="52"/>
+      <c r="N49" s="52"/>
+      <c r="O49" s="54"/>
       <c r="P49" s="6"/>
     </row>
     <row r="50" spans="2:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -1995,6 +1995,30 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="K1:P1"/>
+    <mergeCell ref="C8:O8"/>
+    <mergeCell ref="C10:O10"/>
+    <mergeCell ref="C12:O12"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="I33:O33"/>
+    <mergeCell ref="I16:O16"/>
+    <mergeCell ref="I17:O17"/>
+    <mergeCell ref="I18:O18"/>
+    <mergeCell ref="I19:O19"/>
+    <mergeCell ref="I20:O20"/>
+    <mergeCell ref="I21:O21"/>
+    <mergeCell ref="I22:O22"/>
+    <mergeCell ref="I23:O23"/>
+    <mergeCell ref="I24:O24"/>
+    <mergeCell ref="I25:O25"/>
+    <mergeCell ref="I26:O26"/>
+    <mergeCell ref="I32:O32"/>
+    <mergeCell ref="I15:O15"/>
+    <mergeCell ref="I29:O29"/>
+    <mergeCell ref="I30:O30"/>
+    <mergeCell ref="I31:O31"/>
+    <mergeCell ref="I27:O27"/>
+    <mergeCell ref="I28:O28"/>
     <mergeCell ref="I34:O34"/>
     <mergeCell ref="I47:O47"/>
     <mergeCell ref="I48:O48"/>
@@ -2009,30 +2033,6 @@
     <mergeCell ref="I44:O44"/>
     <mergeCell ref="I45:O45"/>
     <mergeCell ref="I46:O46"/>
-    <mergeCell ref="I15:O15"/>
-    <mergeCell ref="I29:O29"/>
-    <mergeCell ref="I30:O30"/>
-    <mergeCell ref="I31:O31"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="I28:O28"/>
-    <mergeCell ref="I33:O33"/>
-    <mergeCell ref="I16:O16"/>
-    <mergeCell ref="I17:O17"/>
-    <mergeCell ref="I18:O18"/>
-    <mergeCell ref="I19:O19"/>
-    <mergeCell ref="I20:O20"/>
-    <mergeCell ref="I21:O21"/>
-    <mergeCell ref="I22:O22"/>
-    <mergeCell ref="I23:O23"/>
-    <mergeCell ref="I24:O24"/>
-    <mergeCell ref="I25:O25"/>
-    <mergeCell ref="I26:O26"/>
-    <mergeCell ref="I32:O32"/>
-    <mergeCell ref="K1:P1"/>
-    <mergeCell ref="C8:O8"/>
-    <mergeCell ref="C10:O10"/>
-    <mergeCell ref="C12:O12"/>
-    <mergeCell ref="I4:K4"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="64" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>